<commit_message>
fix(inventory): supply titanium metal to A1 traction magnets
The A1 magnet sensitivity recipe bought TiO2 at its elemental-Ti
equivalent mass. This omitted oxide-to-metal reduction before alloying.
Replace that feed with the existing titanium-metal market, whose
background includes chlorination and Kroll magnesium reduction.

Preserve the measured 0.2/100.1 Ti fraction, 95% fabrication retention,
all other constituents, fabrication energy and end-of-life quantities.
B3, the default grade, has no Ti and is unchanged. Actual A1 procurement
and the remaining alloy/powder/coating steps are still evidence gaps.

Validation: exact XML/import scope and elemental closure; native
linking in 18 available ecoinvent version/system-model configurations;
full-network EF 3.1 comparison (A1 climate +0.183%, default paths unchanged).
Stage only the clean workbook correction; retain all 37 pre-existing
scrap-market edits unchanged and unstaged.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-electric-car-mechanical-powertrain.xlsx
+++ b/premise/data/additional_inventories/lci-electric-car-mechanical-powertrain.xlsx
@@ -3104,7 +3104,9 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>NEODYMIUM REDUCTION COVERAGE, 2026-10-20. Replace only the Nd2O3-equivalent feed by equal contained Nd metal from neodymium production, molten salt electrolysis. The provider has explicit oxide/electrode/fluoride/gas/waste balances and documented engineering assumptions. Existing magnet fractions,95%fabrication retention,15kWh/kg downstream fabrication,other precursors and finalEOL are unchanged. Pr/Tb/Dy/Ho and B/Ca/Ti precursor reduction,alloy/powder process specificity and coating remain separate gaps; this is not a complete industrial magnet inventory.
+          <t>TITANIUM PRECURSOR MANUFACTURE, 2026-10-20. The measured A1 grade contains0.2mass%Ti in its rounded100.1%source ledger. Existing TiO2 feed represented elemental equivalence but omitted oxide-to-metal reduction. Replace that feed by market for titanium,GLO,kilogram at TiO2kg*47.867/(47.867+2*15.999). The native market describes titanium metal made via chlorination to TiCl4 and magnesium reduction/vacuumdistillation in the Kroll process; its background manufacture includes the reduction reagents and wastes. It is a commodity-metal feed reference, not measured A1 manufacturer procurement or extra finished-magnet supply. Do not buy an additional oxide,chloride,Mg charge or aerospace triple-melting route on top. New nominal Ti feed0.00210315999789684kg/kgmagnet, leaving0.001998001998002kgTi after the existing95%magnet retention, exactly0.2/100.1. Keep all other A1 constituents,Ndreduction,15kWh/kgdownstream fabrication and finalEOL unchanged. Default B3 contains no Ti; its recipe,motor/vehicle doses and all per-MJ quantities remain unchanged. This resolves Ti reduction coverage for the A1 sensitivity only; other precursor reduction,alloy/powder/coating and actual-grade/process qualification remain open. Existing supplemental workbook only. All original user scrap-market edits remain unstaged and unchanged.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+NEODYMIUM REDUCTION COVERAGE, 2026-10-20. Replace only the Nd2O3-equivalent feed by equal contained Nd metal from neodymium production, molten salt electrolysis. The provider has explicit oxide/electrode/fluoride/gas/waste balances and documented engineering assumptions. Existing magnet fractions,95%fabrication retention,15kWh/kg downstream fabrication,other precursors and finalEOL are unchanged. Pr/Tb/Dy/Ho and B/Ca/Ti precursor reduction,alloy/powder process specificity and coating remain separate gaps; this is not a complete industrial magnet inventory.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
 Nomenclature revision, 2026-10-19. Former activity name: permanent magnet, measured A1 grade, engineering reference. Former reference product: permanent magnet, measured A1 grade, engineering reference. Activity/product labels and supplier references only; coefficients, formulas, uncertainty, declared output and unit are unchanged. Original engineering assumptions, functional-unit basis and limitations remain below.
 APPROVED TRACTION MAGNET GRADE REFERENCES, issue36, 2026-10-18. Jones etal2025 DOI10.1021/jacs.5c04150 SI TableS2, samplesB3 andA1; Hsieh etal2026 DOI10.1007/s11367-026-02610-7 SI TableS11 PMSM bulk components. Select one measured B3 magnet as engineering composition reference, NOT fleet average from two rotors. B3 masspercent:Nd21.9,Pr7.4,Tb0.5,Ho1.7,Co2.2,B0.9,Al0.2,Ca0.2,Fe64.8,Cu0.2 (sum100);Dy not detected, not proof absolutezero. Separate A1 sensitivity:Nd26.6,Tb0.6,Dy0.5,Ho2.2,Co2.4,B0.9,Al0.2,Ca0.1,Ti0.2,Fe66.2,Cu0.2;rounded source100.1percent, divided by100.1 to resolve rounding. Grade choice has substantialNd/Pr/Dy/Tb/Ho/Co sensitivity; unknown fleet penetration,gradeevolution and coercivity requirements remain gaps. Purchase individual oxide suppliers at stoichiometric containedmetal equivalents Nd2O3,Pr6O11,Tb4O7,Ho2O3,Dy2O3,Coasmetal,othermetals explicitly; B usesboricoxide/Causesquicklime/TiusesTiO2 as supply proxies. Oxide-to-metal reduction/reagents,oxygen/byproduct fate,boron/calciumretention and magnet coating are unresolved manufacturing gaps, not a closed full metallurgical process. Assume95percent magnet-material retention, matching5percentfinishedoffcut treatmentproxy, no recyclingcredit; yield sensitivity85-100percent and15kWh/kgmagnetprocess sensitivity5-30. Wholeoxide feed mass can exceed finishedmagnet mass due to oxygen:do not normalize elementalshares by gross feed mass. New roadmotor uses public PMSM non-magnet proportions20.3kgelectricalsteel,4.8Cu,14.6Al,3.9balance allocatedordinary steel as explicit shaft/bearingproxy. Missing source3.9kg componentbreakdown is not a measured steelrecipe. Keep existing0.03735849kgfinishedmagnet/kgmotor and all vehicle motor masses rather than resize magnetdemand to1.3/44.9kg/kg from a differentmotor. Distribute remainingmass across public non-magnet proportions; electricalsteelexisting3.2percentSi reference. Genericmetalworking+1kWh/kgassembly,100percentmotorassemblyretention. Existing motorsteel/Algrades remainproxies; efficiency/torque/voltage not revalidated. Dedicated name outside genericEVmetaloverlay deliberately fixes this source design over time; avoids aluminum overlay doublecount and Nd-onlyoverwrite. No unsupported future gradelearning; future static-vs-learning comparison remains required. Rewire direct car/truck/bus roadmotor inputs and explicit roadperMJ copies; inductionrail/tram unchanged. Existing sourcevehicle life andMJallocation retained. Native backgroundmotor and genericmagnet supplies remain unchanged for other consumers. Individualoxideproviders keep REidentities visible to containedmetal accounting; no primary/secondary claim.</t>
@@ -3488,15 +3490,15 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>market for titanium dioxide</t>
+          <t>market for titanium</t>
         </is>
       </c>
       <c r="B143">
-        <v>0.0035090745865007443</v>
+        <v>0.00210315999789684</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>RER</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3511,12 +3513,17 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>titanium dioxide</t>
+          <t>titanium</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Nominal titanium metal at the former TiO2 contained-Ti-equivalent dose. The native market includes Kroll reduction via TiCl4/Mg; no duplicate oxide or triple-melting purchase. Retained0.2/100.1massfraction and95%magnet fabrication retention are unchanged.</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>titanium dioxide</t>
+          <t>titanium</t>
         </is>
       </c>
     </row>

</xml_diff>